<commit_message>
V1.0 Limpieza de Datos (se deja espacio a figuras y code fuera)
</commit_message>
<xml_diff>
--- a/Data-Analytics/docs/FLEX DRIVE - Permítenos Conocerte (Final - Pruebas).xlsx
+++ b/Data-Analytics/docs/FLEX DRIVE - Permítenos Conocerte (Final - Pruebas).xlsx
@@ -8,17 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leshi\OneDrive\Escritorio\University\006- Ninth Semester\000- Flex Drive\Flex-Drive\Data-Analytics\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{824423A2-7F69-4A1D-BD86-21C4EE559D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E65C294B-2D2D-4B81-9200-E8A5D8E51817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>

</xml_diff>

<commit_message>
V1.3 - Limpieza y Cadenas de Markov
</commit_message>
<xml_diff>
--- a/Data-Analytics/docs/FLEX DRIVE - Permítenos Conocerte (Final - Pruebas).xlsx
+++ b/Data-Analytics/docs/FLEX DRIVE - Permítenos Conocerte (Final - Pruebas).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leshi\OneDrive\Escritorio\University\006- Ninth Semester\000- Flex Drive\Flex-Drive\Data-Analytics\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E65C294B-2D2D-4B81-9200-E8A5D8E51817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3081EBFE-FCDB-450A-BF9D-2FED478D17F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18478" uniqueCount="1036">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18479" uniqueCount="1036">
   <si>
     <t>Acepto.</t>
   </si>
@@ -3209,7 +3209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3220,6 +3220,7 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4748,6 +4749,9 @@
       <c r="CC4" t="s">
         <v>18</v>
       </c>
+      <c r="CD4" t="s">
+        <v>18</v>
+      </c>
       <c r="CF4" t="s">
         <v>65</v>
       </c>
@@ -5587,6 +5591,9 @@
       <c r="CC11" t="s">
         <v>19</v>
       </c>
+      <c r="CE11" t="s">
+        <v>18</v>
+      </c>
       <c r="CF11" t="s">
         <v>110</v>
       </c>
@@ -37176,9 +37183,7 @@
       <c r="BS225" t="s">
         <v>19</v>
       </c>
-      <c r="BT225" t="s">
-        <v>18</v>
-      </c>
+      <c r="BT225" s="6"/>
       <c r="BU225" t="s">
         <v>636</v>
       </c>
@@ -37210,7 +37215,7 @@
         <v>18</v>
       </c>
       <c r="CE225" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="CG225" t="s">
         <v>29</v>
@@ -50139,7 +50144,7 @@
         <v>26</v>
       </c>
       <c r="BK307" t="s">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="BL307" t="s">
         <v>62</v>
@@ -50157,7 +50162,7 @@
         <v>62</v>
       </c>
       <c r="BQ307" t="s">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="BR307" t="s">
         <v>62</v>
@@ -57419,7 +57424,7 @@
         <v>18</v>
       </c>
       <c r="CE353" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="CF353" t="s">
         <v>879</v>

</xml_diff>